<commit_message>
Reviewed Chapter 1 - checkpoint
</commit_message>
<xml_diff>
--- a/report/Khảo sát mức độ hài lòng - Vai trò Chủ tọa - ConferenceSpace (Responses).xlsx
+++ b/report/Khảo sát mức độ hài lòng - Vai trò Chủ tọa - ConferenceSpace (Responses).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="138">
   <si>
     <t>Timestamp</t>
   </si>
@@ -19,6 +19,15 @@
     <t>Tôi hiểu rằng khảo sát này là tự nguyện và dùng để đánh giá trải nghiệm của tôi với ConferenceSpace.</t>
   </si>
   <si>
+    <t>Tôi muốn thực hiện khảo sát này ẩn danh</t>
+  </si>
+  <si>
+    <t>Vị trí hiện tại của bạn</t>
+  </si>
+  <si>
+    <t>Bạn đã từng làm qua các vị trí chuyên môn liên quan nào</t>
+  </si>
+  <si>
     <t>Bạn đã sử dụng vai trò này trong khoảng bao lâu trước khi trả lời?</t>
   </si>
   <si>
@@ -199,18 +208,27 @@
     <t>Email của bạn</t>
   </si>
   <si>
+    <t>Score</t>
+  </si>
+  <si>
     <t>Column 62</t>
   </si>
   <si>
     <t>Có, tôi đồng ý tiếp tục</t>
   </si>
   <si>
+    <t>Có</t>
+  </si>
+  <si>
+    <t>Giảng viên</t>
+  </si>
+  <si>
+    <t>Area Chair, PC Member</t>
+  </si>
+  <si>
     <t>11-20 phút</t>
   </si>
   <si>
-    <t>Có</t>
-  </si>
-  <si>
     <t>Theo dõi tổng quan hoạt động hội nghị trên dashboard, Thiết lập hoặc xem thông tin hội nghị, Quản lý ngày quan trọng, lời mời nộp bài hoặc ban tổ chức, Tạo hội nghị từ template có sẵn, Xem danh sách bài nộp và trạng thái, Sử dụng hoặc hiểu công cụ AI hỗ trợ phân công, phản biện lại hoặc quyết định</t>
   </si>
   <si>
@@ -250,46 +268,163 @@
     <t>Chắc chắn có</t>
   </si>
   <si>
+    <t>incognito@example.com</t>
+  </si>
+  <si>
+    <t>Sau đại học</t>
+  </si>
+  <si>
+    <t>PC Member</t>
+  </si>
+  <si>
+    <t>5-10 phút</t>
+  </si>
+  <si>
+    <t>Thiết lập hoặc xem thông tin hội nghị, Quản lý ngày quan trọng, lời mời nộp bài hoặc ban tổ chức, Xem gợi ý người phản biện và điểm phù hợp, Kiểm tra thông tin xung đột lợi ích</t>
+  </si>
+  <si>
+    <t>Rất hài lòng</t>
+  </si>
+  <si>
+    <t>Rất khó</t>
+  </si>
+  <si>
+    <t>Khó</t>
+  </si>
+  <si>
+    <t>3 - Bình thường</t>
+  </si>
+  <si>
+    <t>Hoàn toàn đồng ý</t>
+  </si>
+  <si>
+    <t>AI hỗ trợ quyết định hoặc phản biện lại</t>
+  </si>
+  <si>
+    <t>Ít bước thao tác hơn, Thông báo lỗi dễ hiểu hơn, Trạng thái và xác nhận rõ hơn, Giao diện dễ đọc hơn, Giải thích AI rõ hơn</t>
+  </si>
+  <si>
+    <t>Không có điều gì gây khó chịu</t>
+  </si>
+  <si>
+    <t>Có lẽ không</t>
+  </si>
+  <si>
+    <t>Mình thấy phần theo dõi rebuttal và phản hồi của reviewer khá rõ nên chair dễ xử lý hơn.</t>
+  </si>
+  <si>
+    <t>Mình thấy hệ thống nên làm rõ hơn mức độ tin cậy của từng insight để chair biết chỗ nào nên kiểm tra lại.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Thạc sĩ</t>
+  </si>
+  <si>
+    <t>Area Chair</t>
+  </si>
+  <si>
     <t>Dưới 5 phút</t>
   </si>
   <si>
     <t>Quản lý ngày quan trọng, lời mời nộp bài hoặc ban tổ chức, Tạo hội nghị từ template có sẵn, Xem danh sách bài nộp và trạng thái, Xem gợi ý người phản biện và điểm phù hợp, Kiểm tra thông tin xung đột lợi ích, Sử dụng hoặc hiểu công cụ AI hỗ trợ phân công, phản biện lại hoặc quyết định</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>nhbang22@clc.fitus.edu.vn</t>
-  </si>
-  <si>
-    <t>Theo dõi tổng quan hoạt động hội nghị trên dashboard, Tạo hội nghị từ template có sẵn, Theo dõi tiến độ phản biện, Xem gợi ý người phản biện và điểm phù hợp, Kiểm tra thông tin xung đột lợi ích, Sử dụng hoặc hiểu công cụ AI hỗ trợ phân công, phản biện lại hoặc quyết định</t>
-  </si>
-  <si>
-    <t>lnmchau22@clc.fitus.edu.vn</t>
+    <t>Theo dõi tiến độ phản biện</t>
+  </si>
+  <si>
+    <t>Danh sách bài nộp</t>
+  </si>
+  <si>
+    <t>Điều hướng rõ hơn, Ít bước thao tác hơn, Trạng thái và xác nhận rõ hơn, Tốc độ phản hồi nhanh hơn, Giải thích AI rõ hơn, Có thêm bằng chứng hoặc nguồn cho gợi ý AI, Dễ bỏ qua hoặc chỉnh sửa gợi ý AI hơn</t>
+  </si>
+  <si>
+    <t>Không</t>
+  </si>
+  <si>
+    <t>Đánh giá học thuật là vấn đề nhạy cảm</t>
+  </si>
+  <si>
+    <t>Chắc chắn không</t>
+  </si>
+  <si>
+    <t>Cái mình thích là hệ thống giúp mình đỡ bị ngợp khi phải đọc nhiều review dài và khá khác nhau.</t>
+  </si>
+  <si>
+    <t>Điều mình muốn cải thiện là AI phải hiểu đúng trọng số giữa score, confidence và nội dung review thay vì chỉ tóm tắt bề mặt.</t>
   </si>
   <si>
     <t>Hơn 20 phút</t>
   </si>
   <si>
-    <t>Theo dõi tổng quan hoạt động hội nghị trên dashboard, Thiết lập hoặc xem thông tin hội nghị, Quản lý ngày quan trọng, lời mời nộp bài hoặc ban tổ chức, Tạo hội nghị từ template có sẵn, Theo dõi tiến độ phản biện, Xem gợi ý người phản biện và điểm phù hợp, Kiểm tra thông tin xung đột lợi ích</t>
-  </si>
-  <si>
-    <t>homanhdung737@gmail.com</t>
-  </si>
-  <si>
-    <t>5-10 phút</t>
-  </si>
-  <si>
-    <t>Quản lý ngày quan trọng, lời mời nộp bài hoặc ban tổ chức, Theo dõi tiến độ phản biện, Xem gợi ý người phản biện và điểm phù hợp, Kiểm tra thông tin xung đột lợi ích</t>
-  </si>
-  <si>
-    <t>vankhoamac9@gmail.com</t>
-  </si>
-  <si>
-    <t>Xem danh sách bài nộp và trạng thái</t>
-  </si>
-  <si>
-    <t>tienphuongbinhthuan@gmail.com</t>
+    <t>Theo dõi tổng quan hoạt động hội nghị trên dashboard, Tạo hội nghị từ template có sẵn, Xem danh sách bài nộp và trạng thái, Theo dõi tiến độ phản biện, Xem gợi ý người phản biện và điểm phù hợp, Kiểm tra thông tin xung đột lợi ích</t>
+  </si>
+  <si>
+    <t>5 - Rất hài lòng</t>
+  </si>
+  <si>
+    <t>Không đồng ý</t>
+  </si>
+  <si>
+    <t>Tạo hội nghị từ template</t>
+  </si>
+  <si>
+    <t>Quản lý ban tổ chức</t>
+  </si>
+  <si>
+    <t>Điều hướng rõ hơn, Giải thích AI rõ hơn, Không có điều cụ thể</t>
+  </si>
+  <si>
+    <t>Không rõ dữ liệu được sử dụng như thế nào</t>
+  </si>
+  <si>
+    <t>Không chắc</t>
+  </si>
+  <si>
+    <t>Mình hài lòng nhất là ConferenceSpace hỗ trợ chair ra quyết định có cơ sở hơn thay vì phải tự tổng hợp mọi thứ bằng tay.</t>
+  </si>
+  <si>
+    <t>Theo mình, trước khi dùng thực tế, ưu tiên số một vẫn là làm AI support cho chair chính xác, minh bạch và dễ kiểm chứng hơn.</t>
+  </si>
+  <si>
+    <t>Thiết lập hoặc xem thông tin hội nghị, Quản lý ngày quan trọng, lời mời nộp bài hoặc ban tổ chức, Xem danh sách bài nộp và trạng thái, Theo dõi tiến độ phản biện, Xem gợi ý người phản biện và điểm phù hợp, Kiểm tra thông tin xung đột lợi ích, Sử dụng hoặc hiểu công cụ AI hỗ trợ phân công, phản biện lại hoặc quyết định</t>
+  </si>
+  <si>
+    <t>Điều hướng rõ hơn, Thông báo lỗi dễ hiểu hơn, Trạng thái và xác nhận rõ hơn, Tốc độ phản hồi nhanh hơn, Giải thích AI rõ hơn, Có thêm bằng chứng hoặc nguồn cho gợi ý AI</t>
+  </si>
+  <si>
+    <t>Yêu cầu quá nhiều thông tin cá nhân</t>
+  </si>
+  <si>
+    <t>Có lẽ có</t>
+  </si>
+  <si>
+    <t>Theo dõi tổng quan hoạt động hội nghị trên dashboard, Tạo hội nghị từ template có sẵn, Theo dõi tiến độ phản biện</t>
+  </si>
+  <si>
+    <t>Ít bước thao tác hơn, Thông báo lỗi dễ hiểu hơn, Giao diện dễ đọc hơn, Giải thích AI rõ hơn, Có thêm bằng chứng hoặc nguồn cho gợi ý AI, Dễ bỏ qua hoặc chỉnh sửa gợi ý AI hơn</t>
+  </si>
+  <si>
+    <t>AI đưa ra phản hồi quá mạnh hoặc gây áp lực</t>
+  </si>
+  <si>
+    <t>Thiết lập hoặc xem thông tin hội nghị, Xem gợi ý người phản biện và điểm phù hợp</t>
+  </si>
+  <si>
+    <t>Quản lý lời mời nộp bài</t>
+  </si>
+  <si>
+    <t>Tốc độ phản hồi nhanh hơn, Giải thích AI rõ hơn, Dễ bỏ qua hoặc chỉnh sửa gợi ý AI hơn, Không có điều cụ thể</t>
+  </si>
+  <si>
+    <t>Xem gợi ý người phản biện và điểm phù hợp</t>
+  </si>
+  <si>
+    <t>Dễ bỏ qua hoặc chỉnh sửa gợi ý AI hơn</t>
+  </si>
+  <si>
+    <t>Quá nhiều trường bắt buộc</t>
   </si>
 </sst>
 </file>
@@ -326,7 +461,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -346,6 +481,9 @@
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -430,71 +568,75 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:BK7" displayName="Form_Responses" name="Form_Responses" id="1">
-  <tableColumns count="63">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:BO9" displayName="Form_Responses" name="Form_Responses" id="1">
+  <tableColumns count="67">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Tôi hiểu rằng khảo sát này là tự nguyện và dùng để đánh giá trải nghiệm của tôi với ConferenceSpace." id="2"/>
-    <tableColumn name="Bạn đã sử dụng vai trò này trong khoảng bao lâu trước khi trả lời?" id="3"/>
-    <tableColumn name="Trước đây bạn đã từng sử dụng hệ thống nộp bài, phản biện hoặc quản lý hội nghị nào khác chưa?" id="4"/>
-    <tableColumn name="Bạn đã thử những phần nào trong vai trò Chủ tọa?" id="5"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Trải nghiệm tổng thể khi sử dụng ConferenceSpace]" id="6"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Tốc độ hoàn thành tác vụ chính]" id="7"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Độ rõ ràng của bố cục và điều hướng]" id="8"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Độ dễ hiểu của nhãn, nút bấm và thông báo]" id="9"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Mức độ đầy đủ của thông tin được hiển thị]" id="10"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Mức độ tin cậy của trạng thái, xác nhận và phản hồi từ hệ thống]" id="11"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Thiết kế giao diện và khả năng đọc thông tin]" id="12"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Sự phù hợp của hệ thống với quy trình hội nghị học thuật]" id="13"/>
-    <tableColumn name="Các thao tác chính dễ hay khó đối với bạn? [Tìm đúng màn hình hoặc chức năng cần dùng]" id="14"/>
-    <tableColumn name="Các thao tác chính dễ hay khó đối với bạn? [Hiểu bước tiếp theo cần làm]" id="15"/>
-    <tableColumn name="Các thao tác chính dễ hay khó đối với bạn? [Hoàn thành tác vụ mà không cần hướng dẫn thêm]" id="16"/>
-    <tableColumn name="Các thao tác chính dễ hay khó đối với bạn? [Nhận biết lỗi, cảnh báo hoặc trường bắt buộc]" id="17"/>
-    <tableColumn name="Các thao tác chính dễ hay khó đối với bạn? [Quay lại hoặc sửa thông tin khi cần]" id="18"/>
-    <tableColumn name="Nếu phải cho điểm mức độ hài lòng tổng thể, bạn sẽ chọn mức nào?" id="19"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Theo dõi tổng quan hoạt động hội nghị trên dashboard]" id="20"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Thiết lập hoặc xem thông tin hội nghị]" id="21"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Quản lý ngày quan trọng, lời mời nộp bài hoặc ban tổ chức]" id="22"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Tạo hội nghị từ template có sẵn]" id="23"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Xem danh sách bài nộp và trạng thái]" id="24"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Theo dõi tiến độ phản biện]" id="25"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Xem gợi ý người phản biện và điểm phù hợp]" id="26"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Kiểm tra thông tin xung đột lợi ích]" id="27"/>
-    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Sử dụng hoặc hiểu công cụ AI hỗ trợ phân công, phản biện lại hoặc quyết định]" id="28"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Dashboard của chủ tọa tóm tắt tình hình hội nghị rõ ràng.]" id="29"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Các khu vực thiết lập hội nghị được tổ chức dễ hiểu.]" id="30"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Trang bài nộp và phân công giúp tôi nhìn thấy tiến độ phản biện.]" id="31"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Gợi ý người phản biện và điểm phù hợp được trình bày dễ hiểu.]" id="32"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Nền tảng cung cấp đủ bằng chứng để tôi cân nhắc gợi ý người phản biện.]" id="33"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Thông tin xung đột lợi ích hỗ trợ ra quyết định cẩn trọng.]" id="34"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Các công cụ AI hỗ trợ chủ tọa nhưng không thay thế quyết định của con người.]" id="35"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Tôi hiểu mục đích của từng màn hình chính trong vai trò Chủ tọa.]" id="36"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Các thông tin quan trọng được đặt ở vị trí dễ thấy.]" id="37"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Tôi không bị quá tải bởi lượng thông tin trên màn hình.]" id="38"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Các trạng thái, hạn chót và hành động cần làm được thể hiện rõ.]" id="39"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Tôi có thể phục hồi khi nhập sai hoặc chưa chắc cần làm gì tiếp theo.]" id="40"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Ngôn ngữ trong hệ thống phù hợp với người dùng sinh viên.]" id="41"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Tôi sẽ cảm thấy thoải mái khi sử dụng vai trò này trong một môn học hoặc dự án nghiên cứu thực tế.]" id="42"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Tôi nhận biết được khi một tính năng đang sử dụng hỗ trợ từ AI.]" id="43"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Gợi ý của AI được trình bày như sự hỗ trợ, không phải quyết định cuối cùng.]" id="44"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Nền tảng cung cấp đủ lý do hoặc bằng chứng cho gợi ý của AI.]" id="45"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Kết quả từ AI giúp giảm thao tác thủ công hoặc tiết kiệm thời gian.]" id="46"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Cảnh báo hoặc khuyến nghị của AI được viết bằng ngôn ngữ dễ hiểu.]" id="47"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Tôi cảm thấy thoải mái khi bỏ qua hoặc đặt nghi vấn về gợi ý của AI.]" id="48"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Tôi muốn hệ thống hiển thị nguồn, lý do hoặc mức độ tin cậy cho gợi ý AI.]" id="49"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Tôi tin rằng quyết định học thuật cuối cùng vẫn nên do con người kiểm soát.]" id="50"/>
-    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Tôi sẽ tin tưởng AI hơn nếu hệ thống cảnh báo rõ khi kết quả có thể chưa đầy đủ hoặc không chắc chắn.]" id="51"/>
-    <tableColumn name="Tính năng hoặc khu vực nào hữu ích nhất với bạn?" id="52"/>
-    <tableColumn name="Tính năng hoặc khu vực nào cần cải thiện nhất?" id="53"/>
-    <tableColumn name="Điều gì sẽ làm bạn hài lòng hơn với hệ thống?" id="54"/>
-    <tableColumn name="Có phần nào khiến bạn không thoải mái không?" id="55"/>
-    <tableColumn name="Nếu có điều khiến bạn không thoải mái, lý do chính là gì?" id="56"/>
-    <tableColumn name="Bạn có sẵn sàng giới thiệu hệ thống này cho bạn cùng lớp hoặc đồng nghiệp dùng thử không?" id="57"/>
-    <tableColumn name="Điều bạn hài lòng nhất khi sử dụng ConferenceSpace là gì?" id="58"/>
-    <tableColumn name="Điều quan trọng nhất cần cải thiện trước khi dùng trong thực tế là gì?" id="59"/>
-    <tableColumn name="Góp ý khác không bắt buộc" id="60"/>
-    <tableColumn name="Email Address" id="61"/>
-    <tableColumn name="Email của bạn" id="62"/>
-    <tableColumn name="Column 62" id="63"/>
+    <tableColumn name="Tôi muốn thực hiện khảo sát này ẩn danh" id="3"/>
+    <tableColumn name="Vị trí hiện tại của bạn" id="4"/>
+    <tableColumn name="Bạn đã từng làm qua các vị trí chuyên môn liên quan nào" id="5"/>
+    <tableColumn name="Bạn đã sử dụng vai trò này trong khoảng bao lâu trước khi trả lời?" id="6"/>
+    <tableColumn name="Trước đây bạn đã từng sử dụng hệ thống nộp bài, phản biện hoặc quản lý hội nghị nào khác chưa?" id="7"/>
+    <tableColumn name="Bạn đã thử những phần nào trong vai trò Chủ tọa?" id="8"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Trải nghiệm tổng thể khi sử dụng ConferenceSpace]" id="9"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Tốc độ hoàn thành tác vụ chính]" id="10"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Độ rõ ràng của bố cục và điều hướng]" id="11"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Độ dễ hiểu của nhãn, nút bấm và thông báo]" id="12"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Mức độ đầy đủ của thông tin được hiển thị]" id="13"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Mức độ tin cậy của trạng thái, xác nhận và phản hồi từ hệ thống]" id="14"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Thiết kế giao diện và khả năng đọc thông tin]" id="15"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các khía cạnh sau? [Sự phù hợp của hệ thống với quy trình hội nghị học thuật]" id="16"/>
+    <tableColumn name="Các thao tác chính dễ hay khó đối với bạn? [Tìm đúng màn hình hoặc chức năng cần dùng]" id="17"/>
+    <tableColumn name="Các thao tác chính dễ hay khó đối với bạn? [Hiểu bước tiếp theo cần làm]" id="18"/>
+    <tableColumn name="Các thao tác chính dễ hay khó đối với bạn? [Hoàn thành tác vụ mà không cần hướng dẫn thêm]" id="19"/>
+    <tableColumn name="Các thao tác chính dễ hay khó đối với bạn? [Nhận biết lỗi, cảnh báo hoặc trường bắt buộc]" id="20"/>
+    <tableColumn name="Các thao tác chính dễ hay khó đối với bạn? [Quay lại hoặc sửa thông tin khi cần]" id="21"/>
+    <tableColumn name="Nếu phải cho điểm mức độ hài lòng tổng thể, bạn sẽ chọn mức nào?" id="22"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Theo dõi tổng quan hoạt động hội nghị trên dashboard]" id="23"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Thiết lập hoặc xem thông tin hội nghị]" id="24"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Quản lý ngày quan trọng, lời mời nộp bài hoặc ban tổ chức]" id="25"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Tạo hội nghị từ template có sẵn]" id="26"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Xem danh sách bài nộp và trạng thái]" id="27"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Theo dõi tiến độ phản biện]" id="28"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Xem gợi ý người phản biện và điểm phù hợp]" id="29"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Kiểm tra thông tin xung đột lợi ích]" id="30"/>
+    <tableColumn name="Bạn hài lòng ở mức nào với các phần sau trong vai trò Chủ tọa? [Sử dụng hoặc hiểu công cụ AI hỗ trợ phân công, phản biện lại hoặc quyết định]" id="31"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Dashboard của chủ tọa tóm tắt tình hình hội nghị rõ ràng.]" id="32"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Các khu vực thiết lập hội nghị được tổ chức dễ hiểu.]" id="33"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Trang bài nộp và phân công giúp tôi nhìn thấy tiến độ phản biện.]" id="34"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Gợi ý người phản biện và điểm phù hợp được trình bày dễ hiểu.]" id="35"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Nền tảng cung cấp đủ bằng chứng để tôi cân nhắc gợi ý người phản biện.]" id="36"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Thông tin xung đột lợi ích hỗ trợ ra quyết định cẩn trọng.]" id="37"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định sau. [Các công cụ AI hỗ trợ chủ tọa nhưng không thay thế quyết định của con người.]" id="38"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Tôi hiểu mục đích của từng màn hình chính trong vai trò Chủ tọa.]" id="39"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Các thông tin quan trọng được đặt ở vị trí dễ thấy.]" id="40"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Tôi không bị quá tải bởi lượng thông tin trên màn hình.]" id="41"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Các trạng thái, hạn chót và hành động cần làm được thể hiện rõ.]" id="42"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Tôi có thể phục hồi khi nhập sai hoặc chưa chắc cần làm gì tiếp theo.]" id="43"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Ngôn ngữ trong hệ thống phù hợp với người dùng sinh viên.]" id="44"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về khả năng sử dụng sau. [Tôi sẽ cảm thấy thoải mái khi sử dụng vai trò này trong một môn học hoặc dự án nghiên cứu thực tế.]" id="45"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Tôi nhận biết được khi một tính năng đang sử dụng hỗ trợ từ AI.]" id="46"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Gợi ý của AI được trình bày như sự hỗ trợ, không phải quyết định cuối cùng.]" id="47"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Nền tảng cung cấp đủ lý do hoặc bằng chứng cho gợi ý của AI.]" id="48"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Kết quả từ AI giúp giảm thao tác thủ công hoặc tiết kiệm thời gian.]" id="49"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Cảnh báo hoặc khuyến nghị của AI được viết bằng ngôn ngữ dễ hiểu.]" id="50"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Tôi cảm thấy thoải mái khi bỏ qua hoặc đặt nghi vấn về gợi ý của AI.]" id="51"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Tôi muốn hệ thống hiển thị nguồn, lý do hoặc mức độ tin cậy cho gợi ý AI.]" id="52"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Tôi tin rằng quyết định học thuật cuối cùng vẫn nên do con người kiểm soát.]" id="53"/>
+    <tableColumn name="Vui lòng đánh giá các nhận định về AI sau. [Tôi sẽ tin tưởng AI hơn nếu hệ thống cảnh báo rõ khi kết quả có thể chưa đầy đủ hoặc không chắc chắn.]" id="54"/>
+    <tableColumn name="Tính năng hoặc khu vực nào hữu ích nhất với bạn?" id="55"/>
+    <tableColumn name="Tính năng hoặc khu vực nào cần cải thiện nhất?" id="56"/>
+    <tableColumn name="Điều gì sẽ làm bạn hài lòng hơn với hệ thống?" id="57"/>
+    <tableColumn name="Có phần nào khiến bạn không thoải mái không?" id="58"/>
+    <tableColumn name="Nếu có điều khiến bạn không thoải mái, lý do chính là gì?" id="59"/>
+    <tableColumn name="Bạn có sẵn sàng giới thiệu hệ thống này cho bạn cùng lớp hoặc đồng nghiệp dùng thử không?" id="60"/>
+    <tableColumn name="Điều bạn hài lòng nhất khi sử dụng ConferenceSpace là gì?" id="61"/>
+    <tableColumn name="Điều quan trọng nhất cần cải thiện trước khi dùng trong thực tế là gì?" id="62"/>
+    <tableColumn name="Góp ý khác không bắt buộc" id="63"/>
+    <tableColumn name="Email Address" id="64"/>
+    <tableColumn name="Email của bạn" id="65"/>
+    <tableColumn name="Score" id="66"/>
+    <tableColumn name="Column 62" id="67"/>
   </tableColumns>
   <tableStyleInfo name="Form Responses 1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
@@ -702,9 +844,14 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="18.88"/>
-    <col customWidth="1" min="2" max="59" width="37.63"/>
-    <col customWidth="1" min="60" max="60" width="25.0"/>
-    <col customWidth="1" min="61" max="69" width="18.88"/>
+    <col customWidth="1" min="2" max="3" width="37.63"/>
+    <col customWidth="1" min="4" max="4" width="28.13"/>
+    <col customWidth="1" min="5" max="5" width="47.0"/>
+    <col customWidth="1" min="6" max="62" width="37.63"/>
+    <col customWidth="1" min="63" max="63" width="25.0"/>
+    <col customWidth="1" min="64" max="64" width="18.88"/>
+    <col customWidth="1" min="65" max="65" width="21.13"/>
+    <col customWidth="1" min="66" max="73" width="18.88"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
@@ -888,14 +1035,26 @@
       <c r="BH1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="BI1" s="2" t="s">
+      <c r="BI1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="BJ1" s="2" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="BK1" s="2" t="s">
+      <c r="BK1" s="1" t="s">
         <v>62</v>
+      </c>
+      <c r="BL1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="BM1" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="BN1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="BO1" s="2" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
@@ -903,279 +1062,1532 @@
         <v>46173.28380049768</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H2" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="U2" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="V2" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="W2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="X2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="Y2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="Z2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="AB2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="AC2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="AD2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="AE2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="AF2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AG2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AH2" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="AI2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AJ2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AK2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AL2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AM2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AN2" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="AO2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AP2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AQ2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AR2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AT2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AU2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AW2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AX2" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="AY2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AZ2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="BA2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="BB2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="BC2" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="BD2" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="BE2" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="BF2" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="I2" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="R2" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="T2" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="U2" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="V2" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="W2" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="X2" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="Y2" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="Z2" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA2" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AB2" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AC2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AD2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AE2" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AF2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AG2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AH2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AI2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AK2" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AL2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AM2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AN2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AO2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AP2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AQ2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AR2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AS2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AT2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AU2" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AV2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AW2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AX2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AY2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AZ2" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="BA2" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="BB2" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="BC2" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="BD2" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="BE2" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="BF2" s="5"/>
-      <c r="BG2" s="5"/>
-      <c r="BH2" s="5"/>
+      <c r="BG2" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="BH2" s="4" t="s">
+        <v>84</v>
+      </c>
       <c r="BI2" s="5"/>
       <c r="BJ2" s="5"/>
       <c r="BK2" s="5"/>
+      <c r="BL2" s="5"/>
+      <c r="BM2" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN2" s="5"/>
+      <c r="BO2" s="5"/>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="6">
-        <v>46197.54418040509</v>
-      </c>
-      <c r="C3" s="7" t="s">
+        <v>46197.81151818287</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="O3" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="P3" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q3" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="R3" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="S3" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="T3" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="U3" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="V3" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="W3" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="X3" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="Y3" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="Z3" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA3" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="AB3" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AC3" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD3" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AE3" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AF3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AG3" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AH3" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E3" s="7" t="s">
+      <c r="AI3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AJ3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AK3" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AL3" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AM3" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN3" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AO3" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AP3" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ3" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AR3" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AS3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AT3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AU3" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AV3" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW3" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AX3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AY3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AZ3" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="BA3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="BB3" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="BC3" s="7" t="s">
         <v>80</v>
       </c>
+      <c r="BD3" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="BE3" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="BF3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="BG3" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="BH3" s="7" t="s">
+        <v>98</v>
+      </c>
       <c r="BI3" s="7" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="BJ3" s="7" t="s">
-        <v>82</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="BL3" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="BM3" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN3" s="8"/>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="6">
-        <v>46197.58514114583</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>64</v>
+        <v>46197.812994259264</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>68</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>65</v>
+        <v>102</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>83</v>
+        <v>103</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="P4" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q4" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="R4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="S4" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T4" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="U4" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="V4" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="W4" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="X4" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="Y4" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="Z4" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA4" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AB4" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC4" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="AD4" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="AE4" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AF4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AG4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AH4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AI4" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AJ4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AK4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AL4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AM4" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AN4" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AO4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AP4" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AQ4" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AR4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS4" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AT4" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AU4" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AV4" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AW4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AX4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AY4" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AZ4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="BA4" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="BB4" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="BC4" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="BD4" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="BE4" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="BF4" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="BG4" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="BH4" s="7" t="s">
+        <v>111</v>
       </c>
       <c r="BI4" s="7" t="s">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="BJ4" s="7" t="s">
-        <v>84</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="BL4" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="BM4" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN4" s="8"/>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="6">
-        <v>46197.59905427083</v>
-      </c>
-      <c r="C5" s="7" t="s">
+        <v>46197.82264557871</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="P5" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="R5" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="S5" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="T5" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="U5" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="V5" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="W5" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="X5" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="Y5" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="Z5" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA5" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AB5" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC5" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD5" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AE5" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AF5" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AG5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AH5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AI5" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AJ5" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AK5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AL5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AM5" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="AN5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AO5" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AP5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AQ5" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AR5" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AS5" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AT5" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AU5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV5" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AW5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AX5" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AY5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AZ5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="BA5" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="BB5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="BC5" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="BD5" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="BE5" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="BF5" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="BG5" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="BH5" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="BI5" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="BJ5" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="BL5" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="BM5" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="BI5" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="BJ5" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="BN5" s="8"/>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="6">
-        <v>46197.62561826389</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>88</v>
+        <v>46197.83165273148</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>68</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>65</v>
+        <v>102</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="BI6" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="BJ6" s="7" t="s">
-        <v>90</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q6" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="R6" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="S6" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="T6" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="U6" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="V6" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="W6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="X6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="Y6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z6" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AB6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AD6" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AE6" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AF6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AG6" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="AH6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AI6" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AJ6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AK6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AL6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AM6" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AN6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AO6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AP6" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AQ6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AR6" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS6" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AT6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AU6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AV6" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AW6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AX6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AY6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AZ6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="BA6" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="BB6" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="BC6" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="BD6" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="BE6" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="BF6" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="BG6" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="BH6" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL6" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="BM6" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN6" s="8"/>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="6">
-        <v>46197.64278672454</v>
-      </c>
-      <c r="C7" s="7" t="s">
+        <v>46197.83442774306</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F7" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E7" s="7" t="s">
+      <c r="G7" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="O7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="P7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="R7" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="S7" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="T7" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="U7" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="BI7" s="7" t="s">
+      <c r="V7" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="W7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="X7" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="Y7" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z7" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="AA7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AB7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AC7" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AD7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AE7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AF7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AG7" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AH7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AI7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AJ7" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AK7" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="AL7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AM7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AN7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AO7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AP7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AR7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AS7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AT7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AU7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AV7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AW7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AX7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AY7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AZ7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="BA7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="BB7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="BC7" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="BD7" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="BJ7" s="7" t="s">
-        <v>92</v>
-      </c>
+      <c r="BE7" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="BF7" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="BG7" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="BH7" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL7" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="BM7" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN7" s="8"/>
+    </row>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="6">
+        <v>46197.84831274305</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="N8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="P8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q8" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="R8" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="S8" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="T8" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="U8" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="V8" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="W8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="X8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="Y8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="Z8" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AB8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AC8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD8" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AE8" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="AF8" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="AG8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AH8" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AI8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AJ8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AK8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AL8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AM8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AO8" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AP8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ8" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AR8" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AT8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AU8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AV8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AW8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AX8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AY8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AZ8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="BA8" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="BB8" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="BC8" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="BD8" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="BE8" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="BF8" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="BG8" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="BH8" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="BL8" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="BM8" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN8" s="8"/>
+    </row>
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="6">
+        <v>46197.850405289355</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="N9" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="O9" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="P9" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="R9" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="S9" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="T9" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="U9" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="V9" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="W9" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="X9" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="Y9" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z9" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA9" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AB9" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AC9" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD9" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AE9" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AF9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AG9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AH9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AI9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AJ9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AK9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AL9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AM9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AO9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AP9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ9" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AR9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AS9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AT9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AU9" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV9" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="AW9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AX9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AY9" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="AZ9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="BA9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="BB9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="BC9" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="BD9" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="BE9" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="BF9" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="BG9" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="BH9" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="BL9" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="BM9" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN9" s="8"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>